<commit_message>
feat: sync Key Metrics of Marketing (1).xlsx with 9-Oct weekly metrics
</commit_message>
<xml_diff>
--- a/public/master/Key Metrics of Marketing (1).xlsx
+++ b/public/master/Key Metrics of Marketing (1).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BD37"/>
+  <dimension ref="A1:BE37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -568,6 +568,9 @@
       <c r="BD1" t="str">
         <v>2-Oct</v>
       </c>
+      <c r="BE1" t="str">
+        <v>9-Oct</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -738,6 +741,9 @@
       <c r="BD2" t="str">
         <v>1.2K</v>
       </c>
+      <c r="BE2" t="str">
+        <v>1.2K</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
@@ -905,6 +911,9 @@
       <c r="BD3">
         <v>856</v>
       </c>
+      <c r="BE3">
+        <v>810</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="str">
@@ -1072,6 +1081,9 @@
       <c r="BD4">
         <v>0.7853</v>
       </c>
+      <c r="BE4">
+        <v>0.7855</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="str">
@@ -1239,6 +1251,9 @@
       <c r="BD5">
         <v>4</v>
       </c>
+      <c r="BE5">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="str">
@@ -1406,6 +1421,9 @@
       <c r="BD6">
         <v>15</v>
       </c>
+      <c r="BE6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
@@ -1573,6 +1591,9 @@
       <c r="BD7">
         <v>0</v>
       </c>
+      <c r="BE7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
@@ -1740,6 +1761,9 @@
       <c r="BD8">
         <v>0</v>
       </c>
+      <c r="BE8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="str">
@@ -1907,6 +1931,9 @@
       <c r="BD9">
         <v>29</v>
       </c>
+      <c r="BE9">
+        <v>29</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="str">
@@ -2074,6 +2101,9 @@
       <c r="BD10">
         <v>18</v>
       </c>
+      <c r="BE10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="str">
@@ -2241,6 +2271,9 @@
       <c r="BD11" t="str">
         <v>1000 (608, 403)</v>
       </c>
+      <c r="BE11" t="str">
+        <v>1400 (951, 410)</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="str">
@@ -2336,6 +2369,9 @@
       <c r="BD12" t="str">
         <v>0, 0, 27</v>
       </c>
+      <c r="BE12" t="str">
+        <v>0, 0, 24</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2613,6 +2649,9 @@
       <c r="BD21">
         <v>4</v>
       </c>
+      <c r="BE21">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="B22" t="str">
@@ -2780,6 +2819,9 @@
       <c r="BD22">
         <v>0</v>
       </c>
+      <c r="BE22">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2950,6 +2992,9 @@
       <c r="BD24">
         <v>4</v>
       </c>
+      <c r="BE24">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="B25" t="str">
@@ -3108,6 +3153,9 @@
       <c r="BD25">
         <v>0</v>
       </c>
+      <c r="BE25">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="B26" t="str">
@@ -3227,6 +3275,9 @@
       <c r="BD26">
         <v>40</v>
       </c>
+      <c r="BE26">
+        <v>3</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" t="str">
@@ -3346,6 +3397,9 @@
       <c r="BD27">
         <v>136</v>
       </c>
+      <c r="BE27">
+        <v>10</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3516,6 +3570,9 @@
       <c r="BD28">
         <v>0</v>
       </c>
+      <c r="BE28">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" t="str">
@@ -3857,7 +3914,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BD37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BE37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>